<commit_message>
feat: ui improvements and field updates
</commit_message>
<xml_diff>
--- a/client/public/templates/Edit_agendamentos.xlsx
+++ b/client/public/templates/Edit_agendamentos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ScopeSystem\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C818BD1-38B3-4BB4-B9FA-8A46533E191D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C2861F4-B40E-4535-9139-AEF0B5C29C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -51,9 +51,6 @@
     <t>Observações</t>
   </si>
   <si>
-    <t>9BD341ACZRY920097</t>
-  </si>
-  <si>
     <t>concluido</t>
   </si>
   <si>
@@ -70,6 +67,9 @@
   </si>
   <si>
     <t>mp</t>
+  </si>
+  <si>
+    <t>9BWBH6BF3T4055034</t>
   </si>
 </sst>
 </file>
@@ -92,9 +92,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="7"/>
-      <color theme="1"/>
-      <name val="Segoe UI"/>
+      <sz val="14"/>
+      <color rgb="FF1D2530"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -136,8 +136,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="40% - Ênfase3" xfId="2" builtinId="39"/>
@@ -456,30 +456,30 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:8" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="3">
+        <v>46073</v>
+      </c>
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="4">
-        <v>46073</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>